<commit_message>
Functional Deeper Dev Milestone 5. Next is refinement for minimal functionality demo.
</commit_message>
<xml_diff>
--- a/tracker/static/tracker/task_import_template.xlsx
+++ b/tracker/static/tracker/task_import_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\frige\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\frige\PycharmProjects\task-tracker\tracker\static\tracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54056ADD-A5EA-43AE-9CEF-47FC48D3F607}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E19664F-A483-451A-8F7A-5D9CAD52AA12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="7830" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tasks" sheetId="1" r:id="rId1"/>
@@ -161,7 +161,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="38">
   <si>
     <t>Task Import Template</t>
   </si>
@@ -276,129 +276,6 @@
   <si>
     <t>Chores</t>
   </si>
-  <si>
-    <t>Test Task 1</t>
-  </si>
-  <si>
-    <t>Pick up groceries after work (don’t forget milk and eggs)</t>
-  </si>
-  <si>
-    <t>Test Task 2</t>
-  </si>
-  <si>
-    <t>Call doctor’s office to reschedule appointment</t>
-  </si>
-  <si>
-    <t>Test Task 3</t>
-  </si>
-  <si>
-    <t>Follow up with Sarah about weekend plans</t>
-  </si>
-  <si>
-    <t>Test Task 4</t>
-  </si>
-  <si>
-    <t>Start laundry before dinner</t>
-  </si>
-  <si>
-    <t>Test Task 5</t>
-  </si>
-  <si>
-    <t>Pay electric bill before due date</t>
-  </si>
-  <si>
-    <t>Test Task 6</t>
-  </si>
-  <si>
-    <t>Clean out fridge and throw away expired food</t>
-  </si>
-  <si>
-    <t>Test Task 7</t>
-  </si>
-  <si>
-    <t>Water plants in the living room</t>
-  </si>
-  <si>
-    <t>Test Task 8</t>
-  </si>
-  <si>
-    <t>Take dog for a longer walk today</t>
-  </si>
-  <si>
-    <t>Test Task 9</t>
-  </si>
-  <si>
-    <t>School</t>
-  </si>
-  <si>
-    <t>Prep lunches for the next couple of days</t>
-  </si>
-  <si>
-    <t>Test Task 10</t>
-  </si>
-  <si>
-    <t>Check calendar and plan out the week</t>
-  </si>
-  <si>
-    <t>Test Task 11</t>
-  </si>
-  <si>
-    <t>Send birthday message to Mike</t>
-  </si>
-  <si>
-    <t>Test Task 12</t>
-  </si>
-  <si>
-    <t>Organize desk and get rid of clutter</t>
-  </si>
-  <si>
-    <t>Test Task 13</t>
-  </si>
-  <si>
-    <t>Look into booking summer vacation</t>
-  </si>
-  <si>
-    <t>Test Task 14</t>
-  </si>
-  <si>
-    <t>Finish reading current book</t>
-  </si>
-  <si>
-    <t>Test Task 15</t>
-  </si>
-  <si>
-    <t>Try new recipe for dinner tonight</t>
-  </si>
-  <si>
-    <t>Test Task 16</t>
-  </si>
-  <si>
-    <t>Set aside time to work out</t>
-  </si>
-  <si>
-    <t>Test Task 17</t>
-  </si>
-  <si>
-    <t>Back up photos from phone</t>
-  </si>
-  <si>
-    <t>Test Task 18</t>
-  </si>
-  <si>
-    <t>Return package at the post office</t>
-  </si>
-  <si>
-    <t>Test Task 19</t>
-  </si>
-  <si>
-    <t>Make list of things needed for the house</t>
-  </si>
-  <si>
-    <t>Test Task 20</t>
-  </si>
-  <si>
-    <t>Relax and take a break — no work tonight</t>
-  </si>
 </sst>
 </file>
 
@@ -491,6 +368,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -498,8 +377,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -816,30 +693,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="18" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
@@ -871,583 +748,154 @@
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="9">
-        <v>46160</v>
-      </c>
-      <c r="D4" s="10">
-        <v>46129.385416666664</v>
-      </c>
-      <c r="E4" s="10"/>
-      <c r="F4">
-        <v>3</v>
-      </c>
-      <c r="G4">
-        <v>6</v>
-      </c>
-      <c r="H4" t="s">
-        <v>39</v>
-      </c>
-      <c r="I4" t="b">
-        <v>0</v>
-      </c>
+      <c r="C4" s="6"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>40</v>
-      </c>
-      <c r="B5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="9">
-        <v>46161</v>
-      </c>
-      <c r="D5" s="10">
-        <v>46130.597222222219</v>
-      </c>
-      <c r="E5" s="10">
-        <v>46131.340277777781</v>
-      </c>
-      <c r="F5">
-        <v>4</v>
-      </c>
-      <c r="G5">
-        <v>6</v>
-      </c>
-      <c r="H5" t="s">
-        <v>41</v>
-      </c>
-      <c r="I5" t="b">
-        <v>1</v>
-      </c>
+      <c r="C5" s="6"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>42</v>
-      </c>
-      <c r="B6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="9">
-        <v>46162</v>
-      </c>
-      <c r="D6" s="10">
-        <v>46131.3125</v>
-      </c>
-      <c r="E6" s="10"/>
-      <c r="F6">
-        <v>5</v>
-      </c>
-      <c r="G6">
-        <v>52</v>
-      </c>
-      <c r="H6" t="s">
-        <v>43</v>
-      </c>
-      <c r="I6" t="b">
-        <v>1</v>
-      </c>
+      <c r="C6" s="6"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>44</v>
-      </c>
-      <c r="B7" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="9">
-        <v>46163</v>
-      </c>
-      <c r="D7" s="10">
-        <v>46132.697916666664</v>
-      </c>
-      <c r="E7" s="10">
-        <v>46133.697916666664</v>
-      </c>
-      <c r="F7">
-        <v>6</v>
-      </c>
-      <c r="G7">
-        <v>49</v>
-      </c>
-      <c r="H7" t="s">
-        <v>45</v>
-      </c>
-      <c r="I7" t="b">
-        <v>1</v>
-      </c>
+      <c r="C7" s="6"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>46</v>
-      </c>
-      <c r="B8" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" s="9">
-        <v>46164</v>
-      </c>
-      <c r="D8" s="10">
-        <v>46133.420138888891</v>
-      </c>
-      <c r="E8" s="10"/>
-      <c r="F8">
-        <v>7</v>
-      </c>
-      <c r="G8">
-        <v>25</v>
-      </c>
-      <c r="H8" t="s">
-        <v>47</v>
-      </c>
-      <c r="I8" t="b">
-        <v>0</v>
-      </c>
+      <c r="C8" s="6"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>48</v>
-      </c>
-      <c r="B9" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" s="9">
-        <v>46165</v>
-      </c>
-      <c r="D9" s="10">
-        <v>46134.527777777781</v>
-      </c>
-      <c r="E9" s="10"/>
-      <c r="F9">
-        <v>8</v>
-      </c>
-      <c r="G9">
-        <v>24</v>
-      </c>
-      <c r="H9" t="s">
-        <v>49</v>
-      </c>
-      <c r="I9" t="b">
-        <v>0</v>
-      </c>
+      <c r="C9" s="6"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>50</v>
-      </c>
-      <c r="B10" t="s">
-        <v>30</v>
-      </c>
-      <c r="C10" s="9">
-        <v>46166</v>
-      </c>
-      <c r="D10" s="10">
-        <v>46135.333333333336</v>
-      </c>
-      <c r="E10" s="10"/>
-      <c r="F10">
-        <v>1</v>
-      </c>
-      <c r="G10">
-        <v>37</v>
-      </c>
-      <c r="H10" t="s">
-        <v>51</v>
-      </c>
-      <c r="I10" t="b">
-        <v>0</v>
-      </c>
+      <c r="C10" s="6"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>52</v>
-      </c>
-      <c r="B11" t="s">
-        <v>30</v>
-      </c>
-      <c r="C11" s="9">
-        <v>46167</v>
-      </c>
-      <c r="D11" s="10">
-        <v>46136.756944444445</v>
-      </c>
-      <c r="E11" s="10">
-        <v>46137.284722222219</v>
-      </c>
-      <c r="F11">
-        <v>1</v>
-      </c>
-      <c r="G11">
-        <v>9</v>
-      </c>
-      <c r="H11" t="s">
-        <v>53</v>
-      </c>
-      <c r="I11" t="b">
-        <v>1</v>
-      </c>
+      <c r="C11" s="6"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B12" t="s">
-        <v>55</v>
-      </c>
-      <c r="C12" s="9">
-        <v>46168</v>
-      </c>
-      <c r="D12" s="10">
-        <v>46137.496527777781</v>
-      </c>
-      <c r="E12" s="10"/>
-      <c r="F12">
-        <v>1</v>
-      </c>
-      <c r="G12">
-        <v>18</v>
-      </c>
-      <c r="H12" t="s">
-        <v>56</v>
-      </c>
-      <c r="I12" t="b">
-        <v>1</v>
-      </c>
+      <c r="C12" s="6"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>57</v>
-      </c>
-      <c r="B13" t="s">
-        <v>55</v>
-      </c>
-      <c r="C13" s="9">
-        <v>46169</v>
-      </c>
-      <c r="D13" s="10">
-        <v>46138.649305555555</v>
-      </c>
-      <c r="E13" s="10">
-        <v>46139.708333333336</v>
-      </c>
-      <c r="F13">
-        <v>1</v>
-      </c>
-      <c r="G13">
-        <v>52</v>
-      </c>
-      <c r="H13" t="s">
-        <v>58</v>
-      </c>
-      <c r="I13" t="b">
-        <v>1</v>
-      </c>
+      <c r="C13" s="6"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>59</v>
-      </c>
-      <c r="B14" t="s">
-        <v>55</v>
-      </c>
-      <c r="C14" s="9">
-        <v>46170</v>
-      </c>
-      <c r="D14" s="10">
-        <v>46139.263888888891</v>
-      </c>
-      <c r="E14" s="10"/>
-      <c r="F14">
-        <v>1</v>
-      </c>
-      <c r="G14">
-        <v>50</v>
-      </c>
-      <c r="H14" t="s">
-        <v>60</v>
-      </c>
-      <c r="I14" t="b">
-        <v>0</v>
-      </c>
+      <c r="C14" s="6"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>61</v>
-      </c>
-      <c r="B15" t="s">
-        <v>55</v>
-      </c>
-      <c r="C15" s="9">
-        <v>46171</v>
-      </c>
-      <c r="D15" s="10">
-        <v>46140.552083333336</v>
-      </c>
-      <c r="E15" s="10"/>
-      <c r="F15">
-        <v>1</v>
-      </c>
-      <c r="G15">
-        <v>36</v>
-      </c>
-      <c r="H15" t="s">
-        <v>62</v>
-      </c>
-      <c r="I15" t="b">
-        <v>0</v>
-      </c>
+      <c r="C15" s="6"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>63</v>
-      </c>
-      <c r="B16" t="s">
-        <v>12</v>
-      </c>
-      <c r="C16" s="9">
-        <v>46172</v>
-      </c>
-      <c r="D16" s="10">
-        <v>46141.725694444445</v>
-      </c>
-      <c r="E16" s="10"/>
-      <c r="F16">
-        <v>1</v>
-      </c>
-      <c r="G16">
-        <v>53</v>
-      </c>
-      <c r="H16" t="s">
-        <v>64</v>
-      </c>
-      <c r="I16" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>65</v>
-      </c>
-      <c r="B17" t="s">
-        <v>30</v>
-      </c>
-      <c r="C17" s="9">
-        <v>46173</v>
-      </c>
-      <c r="D17" s="10">
-        <v>46142.409722222219</v>
-      </c>
-      <c r="E17" s="10">
-        <v>46143.427083333336</v>
-      </c>
-      <c r="F17">
-        <v>2</v>
-      </c>
-      <c r="G17">
-        <v>22</v>
-      </c>
-      <c r="H17" t="s">
-        <v>66</v>
-      </c>
-      <c r="I17" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>67</v>
-      </c>
-      <c r="B18" t="s">
-        <v>55</v>
-      </c>
-      <c r="C18" s="9">
-        <v>46174</v>
-      </c>
-      <c r="D18" s="10">
-        <v>46143.586805555555</v>
-      </c>
-      <c r="E18" s="10"/>
-      <c r="G18">
-        <v>2</v>
-      </c>
-      <c r="H18" t="s">
-        <v>68</v>
-      </c>
-      <c r="I18" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>69</v>
-      </c>
-      <c r="C19" s="9">
-        <v>46175</v>
-      </c>
-      <c r="D19" s="10">
-        <v>46144.322916666664</v>
-      </c>
-      <c r="E19" s="10"/>
-      <c r="G19">
-        <v>23</v>
-      </c>
-      <c r="H19" t="s">
-        <v>70</v>
-      </c>
-      <c r="I19" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>71</v>
-      </c>
-      <c r="C20" s="9">
-        <v>46176</v>
-      </c>
-      <c r="D20" s="10">
-        <v>46145.798611111109</v>
-      </c>
-      <c r="E20" s="10"/>
-      <c r="F20">
-        <v>3</v>
-      </c>
-      <c r="G20">
-        <v>17</v>
-      </c>
-      <c r="H20" t="s">
-        <v>72</v>
-      </c>
-      <c r="I20" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>73</v>
-      </c>
-      <c r="C21" s="9">
-        <v>46177</v>
-      </c>
-      <c r="D21" s="10">
-        <v>46146.4375</v>
-      </c>
-      <c r="E21" s="10"/>
-      <c r="F21">
-        <v>2</v>
-      </c>
-      <c r="G21">
-        <v>15</v>
-      </c>
-      <c r="H21" t="s">
-        <v>74</v>
-      </c>
-      <c r="I21" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>75</v>
-      </c>
-      <c r="C22" s="9">
-        <v>46178</v>
-      </c>
-      <c r="D22" s="10">
-        <v>46147.579861111109</v>
-      </c>
-      <c r="E22" s="10"/>
-      <c r="F22">
-        <v>1</v>
-      </c>
-      <c r="G22">
-        <v>7</v>
-      </c>
-      <c r="H22" t="s">
-        <v>76</v>
-      </c>
-      <c r="I22" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>77</v>
-      </c>
-      <c r="C23" s="9">
-        <v>46179</v>
-      </c>
-      <c r="D23" s="10">
-        <v>46148.350694444445</v>
-      </c>
-      <c r="E23" s="10"/>
-      <c r="F23">
-        <v>3</v>
-      </c>
-      <c r="G23">
-        <v>43</v>
-      </c>
-      <c r="H23" t="s">
-        <v>78</v>
-      </c>
-      <c r="I23" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="C16" s="6"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+    </row>
+    <row r="17" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C17" s="6"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+    </row>
+    <row r="18" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C18" s="6"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+    </row>
+    <row r="19" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C19" s="6"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+    </row>
+    <row r="20" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C20" s="6"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+    </row>
+    <row r="21" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C21" s="6"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+    </row>
+    <row r="22" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C22" s="6"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+    </row>
+    <row r="23" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C23" s="6"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
+    </row>
+    <row r="24" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
       <c r="I24" s="2"/>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
       <c r="I25" s="2"/>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
       <c r="I26" s="2"/>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
       <c r="E27" s="2"/>
       <c r="I27" s="2"/>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
       <c r="I28" s="2"/>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
       <c r="I29" s="2"/>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
       <c r="I30" s="2"/>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
       <c r="I31" s="2"/>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
       <c r="E32" s="2"/>

</xml_diff>